<commit_message>
Corregir filtro de anio en formulas de Gastos (columna F en lugar de E)
</commit_message>
<xml_diff>
--- a/Finanzas_Personales.xlsx
+++ b/Finanzas_Personales.xlsx
@@ -1255,7 +1255,7 @@
         <v>6000</v>
       </c>
       <c r="F7" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D7,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D7,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -1282,7 +1282,7 @@
         <v>3000</v>
       </c>
       <c r="F8" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D8,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D8,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G8" s="10">
@@ -1309,7 +1309,7 @@
         <v>2500</v>
       </c>
       <c r="F9" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D9,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D9,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -1336,7 +1336,7 @@
         <v>2000</v>
       </c>
       <c r="F10" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D10,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D10,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G10" s="10">
@@ -1363,7 +1363,7 @@
         <v>4000</v>
       </c>
       <c r="F11" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D11,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D11,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -1390,7 +1390,7 @@
         <v>2000</v>
       </c>
       <c r="F12" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D12,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D12,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G12" s="10">
@@ -1417,7 +1417,7 @@
         <v>1500</v>
       </c>
       <c r="F13" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D13,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D13,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -1435,7 +1435,7 @@
         <v>1500</v>
       </c>
       <c r="F14" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D14,Gastos!$G:$G,$B$3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$B:$B,$D14,Gastos!$G:$G,$B$3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="G14" s="10">
@@ -1483,7 +1483,7 @@
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,1,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,1,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D18" s="9">
@@ -1502,7 +1502,7 @@
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,2,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,2,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D19" s="9">
@@ -1521,7 +1521,7 @@
         <v/>
       </c>
       <c r="C20" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,3,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,3,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D20" s="9">
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="C21" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,4,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,4,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D21" s="9">
@@ -1559,7 +1559,7 @@
         <v/>
       </c>
       <c r="C22" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,5,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,5,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D22" s="9">
@@ -1578,7 +1578,7 @@
         <v/>
       </c>
       <c r="C23" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,6,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,6,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D23" s="9">
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
       <c r="C24" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,7,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,7,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D24" s="9">
@@ -1616,7 +1616,7 @@
         <v/>
       </c>
       <c r="C25" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,8,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,8,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D25" s="9">
@@ -1635,7 +1635,7 @@
         <v/>
       </c>
       <c r="C26" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,9,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,9,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D26" s="9">
@@ -1654,7 +1654,7 @@
         <v/>
       </c>
       <c r="C27" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,10,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,10,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D27" s="9">
@@ -1673,7 +1673,7 @@
         <v/>
       </c>
       <c r="C28" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,11,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,11,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D28" s="9">
@@ -1692,7 +1692,7 @@
         <v/>
       </c>
       <c r="C29" s="9">
-        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,12,Gastos!$E:$E,$B$4)</f>
+        <f>SUMIFS(Gastos!$D:$D,Gastos!$G:$G,12,Gastos!$F:$F,$B$4)</f>
         <v/>
       </c>
       <c r="D29" s="9">

</xml_diff>